<commit_message>
Adopt joint bootstrap prevalence analysis
</commit_message>
<xml_diff>
--- a/data/intermediate/Base_finalA_N_aleatoria_cohorte_actual_semilla_20260923.xlsx
+++ b/data/intermediate/Base_finalA_N_aleatoria_cohorte_actual_semilla_20260923.xlsx
@@ -499,7 +499,7 @@
         <v>49</v>
       </c>
       <c r="B3">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C3">
         <v>12</v>
@@ -522,7 +522,7 @@
         <v>50</v>
       </c>
       <c r="B4">
-        <v>2008</v>
+        <v>1788</v>
       </c>
       <c r="C4">
         <v>1788</v>
@@ -590,7 +590,7 @@
         <v>51</v>
       </c>
       <c r="B5">
-        <v>1717</v>
+        <v>1548</v>
       </c>
       <c r="C5">
         <v>1548</v>
@@ -658,7 +658,7 @@
         <v>52</v>
       </c>
       <c r="B6">
-        <v>1656</v>
+        <v>1476</v>
       </c>
       <c r="C6">
         <v>1476</v>
@@ -726,7 +726,7 @@
         <v>53</v>
       </c>
       <c r="B7">
-        <v>1642</v>
+        <v>1495</v>
       </c>
       <c r="C7">
         <v>1495</v>
@@ -797,7 +797,7 @@
         <v>54</v>
       </c>
       <c r="B8">
-        <v>1551</v>
+        <v>1385</v>
       </c>
       <c r="C8">
         <v>1385</v>
@@ -868,7 +868,7 @@
         <v>55</v>
       </c>
       <c r="B9">
-        <v>1610</v>
+        <v>1461</v>
       </c>
       <c r="C9">
         <v>1461</v>
@@ -939,7 +939,7 @@
         <v>56</v>
       </c>
       <c r="B10">
-        <v>1536</v>
+        <v>1359</v>
       </c>
       <c r="C10">
         <v>1359</v>
@@ -1010,7 +1010,7 @@
         <v>57</v>
       </c>
       <c r="B11">
-        <v>1566</v>
+        <v>1412</v>
       </c>
       <c r="C11">
         <v>1412</v>
@@ -1081,7 +1081,7 @@
         <v>58</v>
       </c>
       <c r="B12">
-        <v>1436</v>
+        <v>1299</v>
       </c>
       <c r="C12">
         <v>1299</v>
@@ -1152,7 +1152,7 @@
         <v>59</v>
       </c>
       <c r="B13">
-        <v>1406</v>
+        <v>1265</v>
       </c>
       <c r="C13">
         <v>1265</v>
@@ -1223,7 +1223,7 @@
         <v>60</v>
       </c>
       <c r="B14">
-        <v>1400</v>
+        <v>1270</v>
       </c>
       <c r="C14">
         <v>1270</v>
@@ -1294,7 +1294,7 @@
         <v>61</v>
       </c>
       <c r="B15">
-        <v>1387</v>
+        <v>1267</v>
       </c>
       <c r="C15">
         <v>1267</v>
@@ -1365,7 +1365,7 @@
         <v>62</v>
       </c>
       <c r="B16">
-        <v>1293</v>
+        <v>1168</v>
       </c>
       <c r="C16">
         <v>1168</v>
@@ -1436,7 +1436,7 @@
         <v>63</v>
       </c>
       <c r="B17">
-        <v>1326</v>
+        <v>1209</v>
       </c>
       <c r="C17">
         <v>1209</v>
@@ -1504,7 +1504,7 @@
         <v>64</v>
       </c>
       <c r="B18">
-        <v>1253</v>
+        <v>1148</v>
       </c>
       <c r="C18">
         <v>1148</v>
@@ -1575,7 +1575,7 @@
         <v>65</v>
       </c>
       <c r="B19">
-        <v>1367</v>
+        <v>1286</v>
       </c>
       <c r="C19">
         <v>1286</v>
@@ -1646,7 +1646,7 @@
         <v>66</v>
       </c>
       <c r="B20">
-        <v>1324</v>
+        <v>1225</v>
       </c>
       <c r="C20">
         <v>1225</v>
@@ -1717,7 +1717,7 @@
         <v>67</v>
       </c>
       <c r="B21">
-        <v>1274</v>
+        <v>1183</v>
       </c>
       <c r="C21">
         <v>1183</v>
@@ -1785,7 +1785,7 @@
         <v>68</v>
       </c>
       <c r="B22">
-        <v>1234</v>
+        <v>1124</v>
       </c>
       <c r="C22">
         <v>1124</v>
@@ -1856,7 +1856,7 @@
         <v>69</v>
       </c>
       <c r="B23">
-        <v>1147</v>
+        <v>1076</v>
       </c>
       <c r="C23">
         <v>1076</v>
@@ -1927,7 +1927,7 @@
         <v>70</v>
       </c>
       <c r="B24">
-        <v>1154</v>
+        <v>1068</v>
       </c>
       <c r="C24">
         <v>1068</v>
@@ -1998,7 +1998,7 @@
         <v>71</v>
       </c>
       <c r="B25">
-        <v>1031</v>
+        <v>934</v>
       </c>
       <c r="C25">
         <v>934</v>
@@ -2069,7 +2069,7 @@
         <v>72</v>
       </c>
       <c r="B26">
-        <v>883</v>
+        <v>813</v>
       </c>
       <c r="C26">
         <v>813</v>
@@ -2140,7 +2140,7 @@
         <v>73</v>
       </c>
       <c r="B27">
-        <v>817</v>
+        <v>743</v>
       </c>
       <c r="C27">
         <v>743</v>
@@ -2211,7 +2211,7 @@
         <v>74</v>
       </c>
       <c r="B28">
-        <v>735</v>
+        <v>658</v>
       </c>
       <c r="C28">
         <v>658</v>
@@ -2279,7 +2279,7 @@
         <v>75</v>
       </c>
       <c r="B29">
-        <v>488</v>
+        <v>444</v>
       </c>
       <c r="C29">
         <v>444</v>
@@ -2402,7 +2402,7 @@
     </row>
     <row r="32">
       <c r="B32">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C32">
         <v>34</v>

</xml_diff>